<commit_message>
Update hayagsync_staff_import_demo.xlsx with new field and data
</commit_message>
<xml_diff>
--- a/reference_files/hayagsync_staff_import_demo.xlsx
+++ b/reference_files/hayagsync_staff_import_demo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{887FAF14-1698-4463-88A7-BF400E21F7AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CB74865-07C2-404C-869B-9FC68C1379CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="86">
   <si>
     <t>HayagSync Staff ETL Demonstration Template</t>
   </si>
@@ -283,6 +283,15 @@
   </si>
   <si>
     <t>birthdate</t>
+  </si>
+  <si>
+    <t>gender</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Female</t>
   </si>
 </sst>
 </file>
@@ -373,7 +382,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="7">
     <dxf>
       <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -393,6 +402,10 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -407,21 +420,24 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="StaffImportTable" displayName="StaffImportTable" ref="A1:K14" totalsRowShown="0">
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="StaffImportTable" displayName="StaffImportTable" ref="A1:L14" totalsRowShown="0">
+  <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="staff_number"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="first_name"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="last_name"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="middle_name"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="suffix"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="birthdate" dataDxfId="0">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="gender" dataDxfId="6">
       <calculatedColumnFormula>RANDBETWEEN(DATE(1950,1,1), DATE(1999,12,31))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="email" dataDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="phone_number" dataDxfId="4"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="department" dataDxfId="3"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="position_name" dataDxfId="2"/>
-    <tableColumn id="11" xr3:uid="{F60595DE-206A-4328-8A1E-B27D4F03CBC0}" name="employment_status" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="birthdate" dataDxfId="0">
+      <calculatedColumnFormula>RANDBETWEEN(DATE(1950,1,1), DATE(1999,12,31))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="email" dataDxfId="5"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="phone_number" dataDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="department" dataDxfId="3"/>
+    <tableColumn id="11" xr3:uid="{F60595DE-206A-4328-8A1E-B27D4F03CBC0}" name="position_name" dataDxfId="2"/>
+    <tableColumn id="12" xr3:uid="{6A39333F-F27B-4B1E-91C5-2FE76003129B}" name="employment_status" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -708,7 +724,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -723,7 +739,7 @@
     <col min="10" max="10" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="41.4">
+    <row r="1" spans="1:12" ht="41.4">
       <c r="A1" s="3" t="s">
         <v>16</v>
       </c>
@@ -740,25 +756,28 @@
         <v>20</v>
       </c>
       <c r="F1" t="s">
+        <v>83</v>
+      </c>
+      <c r="G1" t="s">
         <v>82</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="27.6">
+    <row r="2" spans="1:12" ht="55.2">
       <c r="A2" s="2" t="s">
         <v>27</v>
       </c>
@@ -770,25 +789,28 @@
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
-      <c r="F2" s="4">
-        <f t="shared" ref="F2:F14" ca="1" si="0">RANDBETWEEN(DATE(1950,1,1), DATE(1999,12,31))</f>
-        <v>24935</v>
-      </c>
-      <c r="G2" s="2" t="s">
+      <c r="F2" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G2" s="4">
+        <f t="shared" ref="G2:G14" ca="1" si="0">RANDBETWEEN(DATE(1950,1,1), DATE(1999,12,31))</f>
+        <v>20628</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="2"/>
+      <c r="J2" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="L2" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="27.6">
+    <row r="3" spans="1:12" ht="55.2">
       <c r="A3" s="2" t="s">
         <v>33</v>
       </c>
@@ -800,25 +822,28 @@
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
-      <c r="F3" s="4">
+      <c r="F3" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="G3" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>20346</v>
-      </c>
-      <c r="G3" s="2" t="s">
+        <v>21228</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="2"/>
+      <c r="J3" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="K3" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="L3" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:12" ht="27.6">
       <c r="A4" s="2" t="s">
         <v>37</v>
       </c>
@@ -830,25 +855,28 @@
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
-      <c r="F4" s="4">
+      <c r="F4" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G4" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>25581</v>
-      </c>
-      <c r="G4" s="2" t="s">
+        <v>32557</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="2"/>
+      <c r="J4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="L4" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:12" ht="27.6">
       <c r="A5" s="2" t="s">
         <v>43</v>
       </c>
@@ -860,25 +888,28 @@
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
-      <c r="F5" s="4">
+      <c r="F5" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="G5" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>26486</v>
-      </c>
-      <c r="G5" s="2" t="s">
+        <v>33945</v>
+      </c>
+      <c r="H5" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2" t="s">
+      <c r="I5" s="2"/>
+      <c r="J5" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="K5" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K5" s="2" t="s">
+      <c r="L5" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:12">
       <c r="A6" s="2" t="s">
         <v>47</v>
       </c>
@@ -890,25 +921,28 @@
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
-      <c r="F6" s="4">
+      <c r="F6" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G6" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>27566</v>
-      </c>
-      <c r="G6" s="2" t="s">
+        <v>32772</v>
+      </c>
+      <c r="H6" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2" t="s">
+      <c r="I6" s="2"/>
+      <c r="J6" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="K6" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="K6" s="2" t="s">
+      <c r="L6" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:12">
       <c r="A7" s="2" t="s">
         <v>53</v>
       </c>
@@ -920,25 +954,28 @@
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
-      <c r="F7" s="4">
+      <c r="F7" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="G7" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>22791</v>
-      </c>
-      <c r="G7" s="2" t="s">
+        <v>33712</v>
+      </c>
+      <c r="H7" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2" t="s">
+      <c r="I7" s="2"/>
+      <c r="J7" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="K7" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="L7" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:12">
       <c r="A8" s="2" t="s">
         <v>57</v>
       </c>
@@ -950,25 +987,28 @@
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
-      <c r="F8" s="4">
+      <c r="F8" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G8" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>22991</v>
-      </c>
-      <c r="G8" s="2" t="s">
+        <v>24313</v>
+      </c>
+      <c r="H8" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2" t="s">
+      <c r="I8" s="2"/>
+      <c r="J8" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="K8" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="L8" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:12">
       <c r="A9" s="2" t="s">
         <v>61</v>
       </c>
@@ -980,25 +1020,28 @@
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
-      <c r="F9" s="4">
+      <c r="F9" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="G9" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>34221</v>
-      </c>
-      <c r="G9" s="2" t="s">
+        <v>19922</v>
+      </c>
+      <c r="H9" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2" t="s">
+      <c r="I9" s="2"/>
+      <c r="J9" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="K9" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="L9" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:12">
       <c r="A10" s="2" t="s">
         <v>65</v>
       </c>
@@ -1010,25 +1053,28 @@
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
-      <c r="F10" s="4">
+      <c r="F10" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G10" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>34862</v>
-      </c>
-      <c r="G10" s="2" t="s">
+        <v>33409</v>
+      </c>
+      <c r="H10" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2" t="s">
+      <c r="I10" s="2"/>
+      <c r="J10" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="K10" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="K10" s="2" t="s">
+      <c r="L10" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:12">
       <c r="A11" s="2" t="s">
         <v>69</v>
       </c>
@@ -1040,25 +1086,28 @@
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
-      <c r="F11" s="4">
+      <c r="F11" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="G11" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>33109</v>
-      </c>
-      <c r="G11" s="2" t="s">
+        <v>20962</v>
+      </c>
+      <c r="H11" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2" t="s">
+      <c r="I11" s="2"/>
+      <c r="J11" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="K11" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="K11" s="2" t="s">
+      <c r="L11" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:12">
       <c r="A12" s="2" t="s">
         <v>73</v>
       </c>
@@ -1070,25 +1119,28 @@
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
-      <c r="F12" s="4">
+      <c r="F12" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G12" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>29075</v>
-      </c>
-      <c r="G12" s="2" t="s">
+        <v>34377</v>
+      </c>
+      <c r="H12" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2" t="s">
+      <c r="I12" s="2"/>
+      <c r="J12" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J12" s="2" t="s">
+      <c r="K12" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="K12" s="2" t="s">
+      <c r="L12" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:12">
       <c r="A13" s="2" t="s">
         <v>77</v>
       </c>
@@ -1100,31 +1152,35 @@
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
-      <c r="F13" s="4">
+      <c r="F13" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G13" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>31011</v>
-      </c>
-      <c r="G13" s="2" t="s">
+        <v>19793</v>
+      </c>
+      <c r="H13" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2" t="s">
+      <c r="I13" s="2"/>
+      <c r="J13" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J13" s="2" t="s">
+      <c r="K13" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="K13" s="2" t="s">
+      <c r="L13" s="2" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:12">
       <c r="F14" s="4"/>
-      <c r="G14" s="2"/>
+      <c r="G14" s="4"/>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Revert "Update hayagsync_staff_import_demo.xlsx with new field and data"
This reverts commit 1c239175174f33f9d91a68ffa08a7cb750f6decc.
</commit_message>
<xml_diff>
--- a/reference_files/hayagsync_staff_import_demo.xlsx
+++ b/reference_files/hayagsync_staff_import_demo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CB74865-07C2-404C-869B-9FC68C1379CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{887FAF14-1698-4463-88A7-BF400E21F7AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="83">
   <si>
     <t>HayagSync Staff ETL Demonstration Template</t>
   </si>
@@ -283,15 +283,6 @@
   </si>
   <si>
     <t>birthdate</t>
-  </si>
-  <si>
-    <t>gender</t>
-  </si>
-  <si>
-    <t>Male</t>
-  </si>
-  <si>
-    <t>Female</t>
   </si>
 </sst>
 </file>
@@ -382,7 +373,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="6">
     <dxf>
       <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -402,10 +393,6 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -420,24 +407,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="StaffImportTable" displayName="StaffImportTable" ref="A1:L14" totalsRowShown="0">
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="StaffImportTable" displayName="StaffImportTable" ref="A1:K14" totalsRowShown="0">
+  <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="staff_number"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="first_name"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="last_name"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="middle_name"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="suffix"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="gender" dataDxfId="6">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="birthdate" dataDxfId="0">
       <calculatedColumnFormula>RANDBETWEEN(DATE(1950,1,1), DATE(1999,12,31))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="birthdate" dataDxfId="0">
-      <calculatedColumnFormula>RANDBETWEEN(DATE(1950,1,1), DATE(1999,12,31))</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="email" dataDxfId="5"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="phone_number" dataDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="department" dataDxfId="3"/>
-    <tableColumn id="11" xr3:uid="{F60595DE-206A-4328-8A1E-B27D4F03CBC0}" name="position_name" dataDxfId="2"/>
-    <tableColumn id="12" xr3:uid="{6A39333F-F27B-4B1E-91C5-2FE76003129B}" name="employment_status" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="email" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="phone_number" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="department" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="position_name" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{F60595DE-206A-4328-8A1E-B27D4F03CBC0}" name="employment_status" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -724,7 +708,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -739,7 +723,7 @@
     <col min="10" max="10" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="41.4">
+    <row r="1" spans="1:11" ht="41.4">
       <c r="A1" s="3" t="s">
         <v>16</v>
       </c>
@@ -756,28 +740,25 @@
         <v>20</v>
       </c>
       <c r="F1" t="s">
-        <v>83</v>
-      </c>
-      <c r="G1" t="s">
         <v>82</v>
       </c>
+      <c r="G1" s="3" t="s">
+        <v>21</v>
+      </c>
       <c r="H1" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="L1" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="55.2">
+    <row r="2" spans="1:11" ht="27.6">
       <c r="A2" s="2" t="s">
         <v>27</v>
       </c>
@@ -789,28 +770,25 @@
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
-      <c r="F2" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="G2" s="4">
-        <f t="shared" ref="G2:G14" ca="1" si="0">RANDBETWEEN(DATE(1950,1,1), DATE(1999,12,31))</f>
-        <v>20628</v>
-      </c>
-      <c r="H2" s="2" t="s">
+      <c r="F2" s="4">
+        <f t="shared" ref="F2:F14" ca="1" si="0">RANDBETWEEN(DATE(1950,1,1), DATE(1999,12,31))</f>
+        <v>24935</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="I2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2" t="s">
+        <v>31</v>
+      </c>
       <c r="J2" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="L2" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="55.2">
+    <row r="3" spans="1:11" ht="27.6">
       <c r="A3" s="2" t="s">
         <v>33</v>
       </c>
@@ -822,28 +800,25 @@
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
-      <c r="F3" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="G3" s="4">
+      <c r="F3" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>21228</v>
-      </c>
-      <c r="H3" s="2" t="s">
+        <v>20346</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="I3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2" t="s">
+        <v>31</v>
+      </c>
       <c r="J3" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="L3" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="27.6">
+    <row r="4" spans="1:11">
       <c r="A4" s="2" t="s">
         <v>37</v>
       </c>
@@ -855,28 +830,25 @@
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
-      <c r="F4" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="G4" s="4">
+      <c r="F4" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>32557</v>
-      </c>
-      <c r="H4" s="2" t="s">
+        <v>25581</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="I4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2" t="s">
+        <v>41</v>
+      </c>
       <c r="J4" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="L4" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="27.6">
+    <row r="5" spans="1:11">
       <c r="A5" s="2" t="s">
         <v>43</v>
       </c>
@@ -888,28 +860,25 @@
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
-      <c r="F5" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="G5" s="4">
+      <c r="F5" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>33945</v>
-      </c>
-      <c r="H5" s="2" t="s">
+        <v>26486</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="I5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2" t="s">
+        <v>41</v>
+      </c>
       <c r="J5" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="L5" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:11">
       <c r="A6" s="2" t="s">
         <v>47</v>
       </c>
@@ -921,28 +890,25 @@
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
-      <c r="F6" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="G6" s="4">
+      <c r="F6" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>32772</v>
-      </c>
-      <c r="H6" s="2" t="s">
+        <v>27566</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="I6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="J6" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="L6" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:11">
       <c r="A7" s="2" t="s">
         <v>53</v>
       </c>
@@ -954,28 +920,25 @@
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
-      <c r="F7" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="G7" s="4">
+      <c r="F7" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>33712</v>
-      </c>
-      <c r="H7" s="2" t="s">
+        <v>22791</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="I7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="J7" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="L7" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="1:11">
       <c r="A8" s="2" t="s">
         <v>57</v>
       </c>
@@ -987,28 +950,25 @@
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
-      <c r="F8" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="G8" s="4">
+      <c r="F8" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>24313</v>
-      </c>
-      <c r="H8" s="2" t="s">
+        <v>22991</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="J8" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="L8" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:12">
+    <row r="9" spans="1:11">
       <c r="A9" s="2" t="s">
         <v>61</v>
       </c>
@@ -1020,28 +980,25 @@
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
-      <c r="F9" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="G9" s="4">
+      <c r="F9" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>19922</v>
-      </c>
-      <c r="H9" s="2" t="s">
+        <v>34221</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="I9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="J9" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="L9" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:12">
+    <row r="10" spans="1:11">
       <c r="A10" s="2" t="s">
         <v>65</v>
       </c>
@@ -1053,28 +1010,25 @@
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
-      <c r="F10" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="G10" s="4">
+      <c r="F10" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>33409</v>
-      </c>
-      <c r="H10" s="2" t="s">
+        <v>34862</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="I10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="J10" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="L10" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:12">
+    <row r="11" spans="1:11">
       <c r="A11" s="2" t="s">
         <v>69</v>
       </c>
@@ -1086,28 +1040,25 @@
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
-      <c r="F11" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="G11" s="4">
+      <c r="F11" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>20962</v>
-      </c>
-      <c r="H11" s="2" t="s">
+        <v>33109</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="I11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="J11" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="L11" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:12">
+    <row r="12" spans="1:11">
       <c r="A12" s="2" t="s">
         <v>73</v>
       </c>
@@ -1119,28 +1070,25 @@
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
-      <c r="F12" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="G12" s="4">
+      <c r="F12" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>34377</v>
-      </c>
-      <c r="H12" s="2" t="s">
+        <v>29075</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="I12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="J12" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="L12" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="1:11">
       <c r="A13" s="2" t="s">
         <v>77</v>
       </c>
@@ -1152,35 +1100,31 @@
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
-      <c r="F13" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="G13" s="4">
+      <c r="F13" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>19793</v>
-      </c>
-      <c r="H13" s="2" t="s">
+        <v>31011</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="I13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="J13" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="L13" s="2" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="14" spans="1:12">
+    <row r="14" spans="1:11">
       <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
+      <c r="G14" s="2"/>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update hayagsync_staff_import_demo.xlsx with revised data and structure
</commit_message>
<xml_diff>
--- a/reference_files/hayagsync_staff_import_demo.xlsx
+++ b/reference_files/hayagsync_staff_import_demo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{887FAF14-1698-4463-88A7-BF400E21F7AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CB74865-07C2-404C-869B-9FC68C1379CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="86">
   <si>
     <t>HayagSync Staff ETL Demonstration Template</t>
   </si>
@@ -283,6 +283,15 @@
   </si>
   <si>
     <t>birthdate</t>
+  </si>
+  <si>
+    <t>gender</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Female</t>
   </si>
 </sst>
 </file>
@@ -373,7 +382,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="7">
     <dxf>
       <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -393,6 +402,10 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -407,21 +420,24 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="StaffImportTable" displayName="StaffImportTable" ref="A1:K14" totalsRowShown="0">
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="StaffImportTable" displayName="StaffImportTable" ref="A1:L14" totalsRowShown="0">
+  <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="staff_number"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="first_name"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="last_name"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="middle_name"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="suffix"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="birthdate" dataDxfId="0">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="gender" dataDxfId="6">
       <calculatedColumnFormula>RANDBETWEEN(DATE(1950,1,1), DATE(1999,12,31))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="email" dataDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="phone_number" dataDxfId="4"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="department" dataDxfId="3"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="position_name" dataDxfId="2"/>
-    <tableColumn id="11" xr3:uid="{F60595DE-206A-4328-8A1E-B27D4F03CBC0}" name="employment_status" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="birthdate" dataDxfId="0">
+      <calculatedColumnFormula>RANDBETWEEN(DATE(1950,1,1), DATE(1999,12,31))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="email" dataDxfId="5"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="phone_number" dataDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="department" dataDxfId="3"/>
+    <tableColumn id="11" xr3:uid="{F60595DE-206A-4328-8A1E-B27D4F03CBC0}" name="position_name" dataDxfId="2"/>
+    <tableColumn id="12" xr3:uid="{6A39333F-F27B-4B1E-91C5-2FE76003129B}" name="employment_status" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -708,7 +724,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -723,7 +739,7 @@
     <col min="10" max="10" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="41.4">
+    <row r="1" spans="1:12" ht="41.4">
       <c r="A1" s="3" t="s">
         <v>16</v>
       </c>
@@ -740,25 +756,28 @@
         <v>20</v>
       </c>
       <c r="F1" t="s">
+        <v>83</v>
+      </c>
+      <c r="G1" t="s">
         <v>82</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="27.6">
+    <row r="2" spans="1:12" ht="55.2">
       <c r="A2" s="2" t="s">
         <v>27</v>
       </c>
@@ -770,25 +789,28 @@
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
-      <c r="F2" s="4">
-        <f t="shared" ref="F2:F14" ca="1" si="0">RANDBETWEEN(DATE(1950,1,1), DATE(1999,12,31))</f>
-        <v>24935</v>
-      </c>
-      <c r="G2" s="2" t="s">
+      <c r="F2" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G2" s="4">
+        <f t="shared" ref="G2:G14" ca="1" si="0">RANDBETWEEN(DATE(1950,1,1), DATE(1999,12,31))</f>
+        <v>20628</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="2"/>
+      <c r="J2" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="L2" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="27.6">
+    <row r="3" spans="1:12" ht="55.2">
       <c r="A3" s="2" t="s">
         <v>33</v>
       </c>
@@ -800,25 +822,28 @@
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
-      <c r="F3" s="4">
+      <c r="F3" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="G3" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>20346</v>
-      </c>
-      <c r="G3" s="2" t="s">
+        <v>21228</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="2"/>
+      <c r="J3" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="K3" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="L3" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:12" ht="27.6">
       <c r="A4" s="2" t="s">
         <v>37</v>
       </c>
@@ -830,25 +855,28 @@
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
-      <c r="F4" s="4">
+      <c r="F4" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G4" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>25581</v>
-      </c>
-      <c r="G4" s="2" t="s">
+        <v>32557</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="2"/>
+      <c r="J4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="L4" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:12" ht="27.6">
       <c r="A5" s="2" t="s">
         <v>43</v>
       </c>
@@ -860,25 +888,28 @@
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
-      <c r="F5" s="4">
+      <c r="F5" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="G5" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>26486</v>
-      </c>
-      <c r="G5" s="2" t="s">
+        <v>33945</v>
+      </c>
+      <c r="H5" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2" t="s">
+      <c r="I5" s="2"/>
+      <c r="J5" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="K5" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K5" s="2" t="s">
+      <c r="L5" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:12">
       <c r="A6" s="2" t="s">
         <v>47</v>
       </c>
@@ -890,25 +921,28 @@
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
-      <c r="F6" s="4">
+      <c r="F6" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G6" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>27566</v>
-      </c>
-      <c r="G6" s="2" t="s">
+        <v>32772</v>
+      </c>
+      <c r="H6" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2" t="s">
+      <c r="I6" s="2"/>
+      <c r="J6" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="K6" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="K6" s="2" t="s">
+      <c r="L6" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:12">
       <c r="A7" s="2" t="s">
         <v>53</v>
       </c>
@@ -920,25 +954,28 @@
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
-      <c r="F7" s="4">
+      <c r="F7" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="G7" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>22791</v>
-      </c>
-      <c r="G7" s="2" t="s">
+        <v>33712</v>
+      </c>
+      <c r="H7" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2" t="s">
+      <c r="I7" s="2"/>
+      <c r="J7" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="K7" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="L7" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:12">
       <c r="A8" s="2" t="s">
         <v>57</v>
       </c>
@@ -950,25 +987,28 @@
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
-      <c r="F8" s="4">
+      <c r="F8" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G8" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>22991</v>
-      </c>
-      <c r="G8" s="2" t="s">
+        <v>24313</v>
+      </c>
+      <c r="H8" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2" t="s">
+      <c r="I8" s="2"/>
+      <c r="J8" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="K8" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="L8" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:12">
       <c r="A9" s="2" t="s">
         <v>61</v>
       </c>
@@ -980,25 +1020,28 @@
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
-      <c r="F9" s="4">
+      <c r="F9" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="G9" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>34221</v>
-      </c>
-      <c r="G9" s="2" t="s">
+        <v>19922</v>
+      </c>
+      <c r="H9" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2" t="s">
+      <c r="I9" s="2"/>
+      <c r="J9" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="K9" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="L9" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:12">
       <c r="A10" s="2" t="s">
         <v>65</v>
       </c>
@@ -1010,25 +1053,28 @@
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
-      <c r="F10" s="4">
+      <c r="F10" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G10" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>34862</v>
-      </c>
-      <c r="G10" s="2" t="s">
+        <v>33409</v>
+      </c>
+      <c r="H10" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2" t="s">
+      <c r="I10" s="2"/>
+      <c r="J10" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="K10" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="K10" s="2" t="s">
+      <c r="L10" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:12">
       <c r="A11" s="2" t="s">
         <v>69</v>
       </c>
@@ -1040,25 +1086,28 @@
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
-      <c r="F11" s="4">
+      <c r="F11" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="G11" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>33109</v>
-      </c>
-      <c r="G11" s="2" t="s">
+        <v>20962</v>
+      </c>
+      <c r="H11" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2" t="s">
+      <c r="I11" s="2"/>
+      <c r="J11" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="K11" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="K11" s="2" t="s">
+      <c r="L11" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:12">
       <c r="A12" s="2" t="s">
         <v>73</v>
       </c>
@@ -1070,25 +1119,28 @@
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
-      <c r="F12" s="4">
+      <c r="F12" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G12" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>29075</v>
-      </c>
-      <c r="G12" s="2" t="s">
+        <v>34377</v>
+      </c>
+      <c r="H12" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2" t="s">
+      <c r="I12" s="2"/>
+      <c r="J12" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J12" s="2" t="s">
+      <c r="K12" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="K12" s="2" t="s">
+      <c r="L12" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:12">
       <c r="A13" s="2" t="s">
         <v>77</v>
       </c>
@@ -1100,31 +1152,35 @@
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
-      <c r="F13" s="4">
+      <c r="F13" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G13" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>31011</v>
-      </c>
-      <c r="G13" s="2" t="s">
+        <v>19793</v>
+      </c>
+      <c r="H13" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2" t="s">
+      <c r="I13" s="2"/>
+      <c r="J13" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J13" s="2" t="s">
+      <c r="K13" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="K13" s="2" t="s">
+      <c r="L13" s="2" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:12">
       <c r="F14" s="4"/>
-      <c r="G14" s="2"/>
+      <c r="G14" s="4"/>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Reimplement AI Analysis and Recommendation feature with temporary fake data for testing; Other minor fixes
</commit_message>
<xml_diff>
--- a/reference_files/hayagsync_staff_import_demo.xlsx
+++ b/reference_files/hayagsync_staff_import_demo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CB74865-07C2-404C-869B-9FC68C1379CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACBFC267-C9B6-4193-855C-BAC0ED100A0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="85">
   <si>
     <t>HayagSync Staff ETL Demonstration Template</t>
   </si>
@@ -129,9 +129,6 @@
     <t>maria.santos@neu.edu.ph</t>
   </si>
   <si>
-    <t>Student Affairs</t>
-  </si>
-  <si>
     <t>Ministrong Tagasubaybay</t>
   </si>
   <si>
@@ -159,9 +156,6 @@
     <t>patricia.garcia@neu.edu.ph</t>
   </si>
   <si>
-    <t>OSD</t>
-  </si>
-  <si>
     <t>OSD Officer</t>
   </si>
   <si>
@@ -189,9 +183,6 @@
     <t>angela.flores@neu.edu.ph</t>
   </si>
   <si>
-    <t>Junior High School</t>
-  </si>
-  <si>
     <t>Teacher</t>
   </si>
   <si>
@@ -292,6 +283,12 @@
   </si>
   <si>
     <t>Female</t>
+  </si>
+  <si>
+    <t>Integrated School</t>
+  </si>
+  <si>
+    <t>Office of Student Discipline</t>
   </si>
 </sst>
 </file>
@@ -384,7 +381,6 @@
   </cellStyles>
   <dxfs count="7">
     <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -400,6 +396,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -430,14 +427,14 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="gender" dataDxfId="6">
       <calculatedColumnFormula>RANDBETWEEN(DATE(1950,1,1), DATE(1999,12,31))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="birthdate" dataDxfId="0">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="birthdate" dataDxfId="5">
       <calculatedColumnFormula>RANDBETWEEN(DATE(1950,1,1), DATE(1999,12,31))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="email" dataDxfId="5"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="phone_number" dataDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="department" dataDxfId="3"/>
-    <tableColumn id="11" xr3:uid="{F60595DE-206A-4328-8A1E-B27D4F03CBC0}" name="position_name" dataDxfId="2"/>
-    <tableColumn id="12" xr3:uid="{6A39333F-F27B-4B1E-91C5-2FE76003129B}" name="employment_status" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="email" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="phone_number" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="department" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{F60595DE-206A-4328-8A1E-B27D4F03CBC0}" name="position_name" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{6A39333F-F27B-4B1E-91C5-2FE76003129B}" name="employment_status" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -756,10 +753,10 @@
         <v>20</v>
       </c>
       <c r="F1" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="G1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>21</v>
@@ -790,21 +787,21 @@
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="G2" s="4">
-        <f t="shared" ref="G2:G14" ca="1" si="0">RANDBETWEEN(DATE(1950,1,1), DATE(1999,12,31))</f>
-        <v>20628</v>
+        <f t="shared" ref="G2:G13" ca="1" si="0">RANDBETWEEN(DATE(1950,1,1), DATE(1999,12,31))</f>
+        <v>21750</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>30</v>
       </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="K2" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>32</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>26</v>
@@ -812,32 +809,32 @@
     </row>
     <row r="3" spans="1:12" ht="55.2">
       <c r="A3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>35</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="4" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="G3" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>21228</v>
+        <v>27046</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="K3" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>32</v>
       </c>
       <c r="L3" s="2" t="s">
         <v>26</v>
@@ -845,32 +842,32 @@
     </row>
     <row r="4" spans="1:12" ht="27.6">
       <c r="A4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="G4" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>32557</v>
+        <v>28881</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2" t="s">
-        <v>41</v>
+        <v>84</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="L4" s="2" t="s">
         <v>26</v>
@@ -878,32 +875,32 @@
     </row>
     <row r="5" spans="1:12" ht="27.6">
       <c r="A5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>45</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="4" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="G5" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>33945</v>
+        <v>23459</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2" t="s">
-        <v>41</v>
+        <v>84</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="L5" s="2" t="s">
         <v>26</v>
@@ -911,32 +908,32 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>49</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="G6" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>32772</v>
+        <v>19641</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2" t="s">
-        <v>51</v>
+        <v>83</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>26</v>
@@ -944,32 +941,32 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7" s="2" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="4" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="G7" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>33712</v>
+        <v>34465</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2" t="s">
-        <v>51</v>
+        <v>83</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="L7" s="2" t="s">
         <v>26</v>
@@ -977,32 +974,32 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="G8" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>24313</v>
+        <v>21100</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2" t="s">
-        <v>51</v>
+        <v>83</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="L8" s="2" t="s">
         <v>26</v>
@@ -1010,32 +1007,32 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="4" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="G9" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>19922</v>
+        <v>29789</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2" t="s">
-        <v>51</v>
+        <v>83</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="L9" s="2" t="s">
         <v>26</v>
@@ -1043,32 +1040,32 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10" s="2" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="G10" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>33409</v>
+        <v>22638</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2" t="s">
-        <v>51</v>
+        <v>83</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="L10" s="2" t="s">
         <v>26</v>
@@ -1076,32 +1073,32 @@
     </row>
     <row r="11" spans="1:12">
       <c r="A11" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="F11" s="4" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="G11" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>20962</v>
+        <v>22027</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2" t="s">
-        <v>51</v>
+        <v>83</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="L11" s="2" t="s">
         <v>26</v>
@@ -1109,32 +1106,32 @@
     </row>
     <row r="12" spans="1:12">
       <c r="A12" s="2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="G12" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>34377</v>
+        <v>35759</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="I12" s="2"/>
       <c r="J12" s="2" t="s">
-        <v>51</v>
+        <v>83</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="L12" s="2" t="s">
         <v>26</v>
@@ -1142,35 +1139,35 @@
     </row>
     <row r="13" spans="1:12">
       <c r="A13" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="G13" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>19793</v>
+        <v>19847</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="I13" s="2"/>
       <c r="J13" s="2" t="s">
-        <v>51</v>
+        <v>83</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:12">

</xml_diff>